<commit_message>
Keepers: live MLB team affiliations (0 blanks, warehouse-sourced)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/LPT-Keeper-Status-2026.xlsx
+++ b/downloads/LPT-Keeper-Status-2026.xlsx
@@ -669,7 +669,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>LAA</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
@@ -735,7 +735,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>SFG</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>LAA</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>CHW</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
@@ -1228,7 +1228,11 @@
           <t>C. Encarnacion-Strand</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>BAL</t>
+        </is>
+      </c>
       <c r="E24" s="2" t="n">
         <v>2</v>
       </c>
@@ -1523,7 +1527,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>CHW</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
@@ -1556,7 +1560,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>TBR</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
@@ -1754,7 +1758,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>WSN</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -1787,7 +1791,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>KCR</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -1985,7 +1989,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>KCR</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -2018,7 +2022,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>BAL</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -2084,7 +2088,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>SDP</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E50" t="n">
@@ -2150,7 +2154,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>TBR</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E52" t="n">
@@ -2282,7 +2286,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>WSN</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="E56" t="n">
@@ -2348,7 +2352,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>WSN</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -2445,7 +2449,11 @@
           <t>Vaughn Grissom</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>LAA</t>
+        </is>
+      </c>
       <c r="E61" t="n">
         <v>1</v>
       </c>
@@ -2573,7 +2581,11 @@
           <t>Cody Bradford</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr"/>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>TEX</t>
+        </is>
+      </c>
       <c r="E65" t="n">
         <v>1</v>
       </c>
@@ -2934,7 +2946,7 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>TBR</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E76" s="2" t="n">
@@ -3033,7 +3045,7 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>KCR</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="E79" s="2" t="n">
@@ -3198,7 +3210,7 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>SFG</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="E84" s="2" t="n">
@@ -3231,7 +3243,7 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>WSN</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="E85" s="2" t="n">
@@ -3594,7 +3606,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>SFG</t>
+          <t>PHI</t>
         </is>
       </c>
       <c r="E96" s="2" t="n">
@@ -3660,7 +3672,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>KCR</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="E98" s="2" t="n">
@@ -3792,7 +3804,7 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>SDP</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E102" s="2" t="n">
@@ -3825,7 +3837,7 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>WSN</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="E103" s="2" t="n">
@@ -3891,7 +3903,7 @@
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>TBR</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E105" s="2" t="n">
@@ -4023,7 +4035,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="E109" t="n">
@@ -4287,7 +4299,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>TBR</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E117" t="n">
@@ -4320,7 +4332,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>TBR</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E118" t="n">
@@ -4452,7 +4464,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="E122" t="n">
@@ -4518,7 +4530,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>SDP</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E124" t="n">
@@ -4615,7 +4627,11 @@
           <t>Osleivis Basabe</t>
         </is>
       </c>
-      <c r="D127" t="inlineStr"/>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
       <c r="E127" t="n">
         <v>3</v>
       </c>
@@ -4712,7 +4728,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>CIN</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="E130" t="n">
@@ -4745,7 +4761,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>SDP</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E131" t="n">
@@ -4778,7 +4794,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>CHW</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -4811,7 +4827,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>NYM</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="E133" t="n">
@@ -4844,7 +4860,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>NYM</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="E134" t="n">
@@ -4877,7 +4893,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>SDP</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E135" t="n">
@@ -4943,7 +4959,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>TBR</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E137" t="n">
@@ -5108,7 +5124,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>CHW</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E142" t="n">
@@ -5432,7 +5448,11 @@
           <t>Angel Genao</t>
         </is>
       </c>
-      <c r="D152" s="2" t="inlineStr"/>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>CLE</t>
+        </is>
+      </c>
       <c r="E152" s="2" t="n">
         <v>12</v>
       </c>
@@ -5461,7 +5481,11 @@
           <t>George Lombard Jr.</t>
         </is>
       </c>
-      <c r="D153" s="2" t="inlineStr"/>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>NYY</t>
+        </is>
+      </c>
       <c r="E153" s="2" t="n">
         <v>12</v>
       </c>
@@ -5822,7 +5846,7 @@
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>CHW</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="E164" s="2" t="n">
@@ -5954,7 +5978,7 @@
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>SFG</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="E168" s="2" t="n">
@@ -5987,7 +6011,7 @@
       </c>
       <c r="D169" s="2" t="inlineStr">
         <is>
-          <t>KCR</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="E169" s="2" t="n">
@@ -6053,7 +6077,7 @@
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>KCR</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="E171" s="2" t="n">
@@ -6251,7 +6275,7 @@
       </c>
       <c r="D177" s="2" t="inlineStr">
         <is>
-          <t>WSN</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="E177" s="2" t="n">
@@ -6449,7 +6473,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>KCR</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="E183" t="n">
@@ -6482,7 +6506,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>SFG</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="E184" t="n">
@@ -6515,7 +6539,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>SFG</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="E185" t="n">
@@ -6746,7 +6770,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>BAL</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="E192" t="n">
@@ -7041,7 +7065,11 @@
           <t>Tyler Wells</t>
         </is>
       </c>
-      <c r="D201" t="inlineStr"/>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>TB</t>
+        </is>
+      </c>
       <c r="E201" t="n">
         <v>2</v>
       </c>
@@ -7301,7 +7329,11 @@
           <t>Brent Headrick</t>
         </is>
       </c>
-      <c r="D209" t="inlineStr"/>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>NYY</t>
+        </is>
+      </c>
       <c r="E209" t="n">
         <v>1</v>
       </c>
@@ -7530,7 +7562,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>TBR</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E216" t="n">
@@ -7728,7 +7760,7 @@
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="E222" s="2" t="n">
@@ -7827,7 +7859,7 @@
       </c>
       <c r="D225" s="2" t="inlineStr">
         <is>
-          <t>NYM</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E225" s="2" t="n">
@@ -7926,7 +7958,7 @@
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>CHW</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E228" s="2" t="n">
@@ -7959,7 +7991,7 @@
       </c>
       <c r="D229" s="2" t="inlineStr">
         <is>
-          <t>SDP</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E229" s="2" t="n">
@@ -8190,7 +8222,7 @@
       </c>
       <c r="D236" s="2" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E236" s="2" t="n">
@@ -8388,7 +8420,7 @@
       </c>
       <c r="D242" s="2" t="inlineStr">
         <is>
-          <t>TBR</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E242" s="2" t="n">
@@ -8553,7 +8585,7 @@
       </c>
       <c r="D247" s="2" t="inlineStr">
         <is>
-          <t>KCR</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="E247" s="2" t="n">
@@ -9011,7 +9043,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E261" t="n">
@@ -9242,7 +9274,7 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>KCR</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="E268" t="n">
@@ -9407,7 +9439,7 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>WSN</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="E273" t="n">
@@ -9605,7 +9637,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>TBR</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E279" t="n">
@@ -9638,7 +9670,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>CHW</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E280" t="n">
@@ -9737,7 +9769,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>CHW</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E283" t="n">
@@ -9803,7 +9835,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>TBR</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E285" t="n">
@@ -9935,7 +9967,7 @@
       </c>
       <c r="D289" s="2" t="inlineStr">
         <is>
-          <t>SDP</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E289" s="2" t="n">
@@ -10298,7 +10330,7 @@
       </c>
       <c r="D300" s="2" t="inlineStr">
         <is>
-          <t>TBR</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E300" s="2" t="n">
@@ -10397,7 +10429,7 @@
       </c>
       <c r="D303" s="2" t="inlineStr">
         <is>
-          <t>NYM</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="E303" s="2" t="n">
@@ -10428,7 +10460,11 @@
           <t>Cristian Javier</t>
         </is>
       </c>
-      <c r="D304" s="2" t="inlineStr"/>
+      <c r="D304" s="2" t="inlineStr">
+        <is>
+          <t>HOU</t>
+        </is>
+      </c>
       <c r="E304" s="2" t="n">
         <v>5</v>
       </c>
@@ -10591,7 +10627,7 @@
       </c>
       <c r="D309" s="2" t="inlineStr">
         <is>
-          <t>LAA</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E309" s="2" t="n">
@@ -10723,7 +10759,7 @@
       </c>
       <c r="D313" s="2" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E313" s="2" t="n">
@@ -10756,7 +10792,7 @@
       </c>
       <c r="D314" s="2" t="inlineStr">
         <is>
-          <t>KCR</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="E314" s="2" t="n">
@@ -10822,7 +10858,7 @@
       </c>
       <c r="D316" s="2" t="inlineStr">
         <is>
-          <t>SDP</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E316" s="2" t="n">
@@ -11020,7 +11056,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>SDP</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E322" t="n">
@@ -11515,7 +11551,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>WSN</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="E337" t="n">
@@ -11614,7 +11650,7 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>CHW</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E340" t="n">
@@ -11911,7 +11947,7 @@
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>TBR</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="E349" t="n">
@@ -12307,7 +12343,7 @@
       </c>
       <c r="D361" s="2" t="inlineStr">
         <is>
-          <t>WSN</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="E361" s="2" t="n">
@@ -12472,7 +12508,7 @@
       </c>
       <c r="D366" s="2" t="inlineStr">
         <is>
-          <t>SDP</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E366" s="2" t="n">
@@ -12670,7 +12706,7 @@
       </c>
       <c r="D372" s="2" t="inlineStr">
         <is>
-          <t>KCR</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="E372" s="2" t="n">
@@ -12703,7 +12739,7 @@
       </c>
       <c r="D373" s="2" t="inlineStr">
         <is>
-          <t>SDP</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E373" s="2" t="n">
@@ -12901,7 +12937,7 @@
       </c>
       <c r="D379" s="2" t="inlineStr">
         <is>
-          <t>WSN</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="E379" s="2" t="n">
@@ -13033,7 +13069,7 @@
       </c>
       <c r="D383" s="2" t="inlineStr">
         <is>
-          <t>KCR</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="E383" s="2" t="n">
@@ -13132,7 +13168,7 @@
       </c>
       <c r="D386" s="2" t="inlineStr">
         <is>
-          <t>SDP</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E386" s="2" t="n">
@@ -13196,7 +13232,11 @@
           <t>Victor Mesa Jr.</t>
         </is>
       </c>
-      <c r="D388" s="2" t="inlineStr"/>
+      <c r="D388" s="2" t="inlineStr">
+        <is>
+          <t>TB</t>
+        </is>
+      </c>
       <c r="E388" s="2" t="n">
         <v>1</v>
       </c>
@@ -13355,7 +13395,7 @@
       </c>
       <c r="D393" t="inlineStr">
         <is>
-          <t>SFG</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="E393" t="n">
@@ -13487,7 +13527,7 @@
       </c>
       <c r="D397" t="inlineStr">
         <is>
-          <t>SFG</t>
+          <t>NYY</t>
         </is>
       </c>
       <c r="E397" t="n">
@@ -13553,7 +13593,7 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>HOU</t>
         </is>
       </c>
       <c r="E399" t="n">
@@ -13982,7 +14022,7 @@
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>MIL</t>
         </is>
       </c>
       <c r="E412" t="n">
@@ -14112,7 +14152,11 @@
           <t>Hayden Wesneski</t>
         </is>
       </c>
-      <c r="D416" t="inlineStr"/>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>HOU</t>
+        </is>
+      </c>
       <c r="E416" t="n">
         <v>1</v>
       </c>
@@ -14273,7 +14317,11 @@
           <t>Andruw Monasterio</t>
         </is>
       </c>
-      <c r="D421" t="inlineStr"/>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
       <c r="E421" t="n">
         <v>1</v>
       </c>
@@ -14436,7 +14484,7 @@
       </c>
       <c r="D426" s="3" t="inlineStr">
         <is>
-          <t>KCR</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="E426" s="3" t="n">
@@ -14667,7 +14715,7 @@
       </c>
       <c r="D433" s="3" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E433" s="3" t="n">
@@ -14931,7 +14979,7 @@
       </c>
       <c r="D441" s="3" t="inlineStr">
         <is>
-          <t>SFG</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="E441" s="3" t="n">
@@ -15096,7 +15144,7 @@
       </c>
       <c r="D446" s="3" t="inlineStr">
         <is>
-          <t>CHW</t>
+          <t>CWS</t>
         </is>
       </c>
       <c r="E446" s="3" t="n">
@@ -15129,7 +15177,7 @@
       </c>
       <c r="D447" s="3" t="inlineStr">
         <is>
-          <t>WSN</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E447" s="3" t="n">
@@ -15195,7 +15243,7 @@
       </c>
       <c r="D449" s="3" t="inlineStr">
         <is>
-          <t>SDP</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E449" s="3" t="n">
@@ -15459,7 +15507,7 @@
       </c>
       <c r="D457" s="3" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>ARI</t>
         </is>
       </c>
       <c r="E457" s="3" t="n">
@@ -15657,7 +15705,7 @@
       </c>
       <c r="D463" s="3" t="inlineStr">
         <is>
-          <t>WSN</t>
+          <t>ARI</t>
         </is>
       </c>
       <c r="E463" s="3" t="n">
@@ -15690,7 +15738,7 @@
       </c>
       <c r="D464" s="3" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E464" s="3" t="n">
@@ -16449,7 +16497,7 @@
       </c>
       <c r="D487" s="3" t="inlineStr">
         <is>
-          <t>NYM</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="E487" s="3" t="n">
@@ -16482,7 +16530,7 @@
       </c>
       <c r="D488" s="3" t="inlineStr">
         <is>
-          <t>SDP</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E488" s="3" t="n">
@@ -16911,7 +16959,7 @@
       </c>
       <c r="D501" s="3" t="inlineStr">
         <is>
-          <t>BAL</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="E501" s="3" t="n">
@@ -17109,7 +17157,7 @@
       </c>
       <c r="D507" s="3" t="inlineStr">
         <is>
-          <t>KCR</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="E507" s="3" t="n">
@@ -17340,7 +17388,7 @@
       </c>
       <c r="D514" s="3" t="inlineStr">
         <is>
-          <t>KCR</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="E514" s="3" t="n">
@@ -17505,7 +17553,7 @@
       </c>
       <c r="D519" s="3" t="inlineStr">
         <is>
-          <t>SDP</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="E519" s="3" t="n">
@@ -17703,7 +17751,7 @@
       </c>
       <c r="D525" s="3" t="inlineStr">
         <is>
-          <t>ARI</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E525" s="3" t="n">

</xml_diff>

<commit_message>
Keepers: Arias/Hope/Zeferjahn teams resolved (prospect fallback + MLBAM pin)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/LPT-Keeper-Status-2026.xlsx
+++ b/downloads/LPT-Keeper-Status-2026.xlsx
@@ -5188,7 +5188,11 @@
           <t>Franklin Arias</t>
         </is>
       </c>
-      <c r="D144" t="inlineStr"/>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
       <c r="E144" t="n">
         <v>1</v>
       </c>
@@ -8682,7 +8686,11 @@
           <t>Zyhir Hope</t>
         </is>
       </c>
-      <c r="D250" s="2" t="inlineStr"/>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>LAD</t>
+        </is>
+      </c>
       <c r="E250" s="2" t="n">
         <v>1</v>
       </c>
@@ -13298,7 +13306,11 @@
           <t>Ryan Zeferjahn</t>
         </is>
       </c>
-      <c r="D390" s="2" t="inlineStr"/>
+      <c r="D390" s="2" t="inlineStr">
+        <is>
+          <t>CHC</t>
+        </is>
+      </c>
       <c r="E390" s="2" t="n">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Jimmy Bowman -> Jimmy site-wide
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/LPT-Keeper-Status-2026.xlsx
+++ b/downloads/LPT-Keeper-Status-2026.xlsx
@@ -9960,7 +9960,7 @@
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B289" s="2" t="inlineStr">
@@ -9993,7 +9993,7 @@
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B290" s="2" t="inlineStr">
@@ -10026,7 +10026,7 @@
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B291" s="2" t="inlineStr">
@@ -10059,7 +10059,7 @@
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B292" s="2" t="inlineStr">
@@ -10092,7 +10092,7 @@
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B293" s="2" t="inlineStr">
@@ -10125,7 +10125,7 @@
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B294" s="2" t="inlineStr">
@@ -10158,7 +10158,7 @@
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B295" s="2" t="inlineStr">
@@ -10191,7 +10191,7 @@
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B296" s="2" t="inlineStr">
@@ -10224,7 +10224,7 @@
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B297" s="2" t="inlineStr">
@@ -10257,7 +10257,7 @@
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B298" s="2" t="inlineStr">
@@ -10290,7 +10290,7 @@
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B299" s="2" t="inlineStr">
@@ -10323,7 +10323,7 @@
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B300" s="2" t="inlineStr">
@@ -10356,7 +10356,7 @@
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B301" s="2" t="inlineStr">
@@ -10389,7 +10389,7 @@
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B302" s="2" t="inlineStr">
@@ -10422,7 +10422,7 @@
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B303" s="2" t="inlineStr">
@@ -10455,7 +10455,7 @@
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B304" s="2" t="inlineStr">
@@ -10488,7 +10488,7 @@
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B305" s="2" t="inlineStr">
@@ -10521,7 +10521,7 @@
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B306" s="2" t="inlineStr">
@@ -10554,7 +10554,7 @@
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B307" s="2" t="inlineStr">
@@ -10587,7 +10587,7 @@
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B308" s="2" t="inlineStr">
@@ -10620,7 +10620,7 @@
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B309" s="2" t="inlineStr">
@@ -10653,7 +10653,7 @@
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B310" s="2" t="inlineStr">
@@ -10686,7 +10686,7 @@
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B311" s="2" t="inlineStr">
@@ -10719,7 +10719,7 @@
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B312" s="2" t="inlineStr">
@@ -10752,7 +10752,7 @@
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B313" s="2" t="inlineStr">
@@ -10785,7 +10785,7 @@
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B314" s="2" t="inlineStr">
@@ -10818,7 +10818,7 @@
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B315" s="2" t="inlineStr">
@@ -10851,7 +10851,7 @@
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B316" s="2" t="inlineStr">
@@ -10884,7 +10884,7 @@
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B317" s="2" t="inlineStr">
@@ -10917,7 +10917,7 @@
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B318" s="2" t="inlineStr">
@@ -10950,7 +10950,7 @@
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B319" s="2" t="inlineStr">
@@ -10983,7 +10983,7 @@
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B320" s="2" t="inlineStr">
@@ -11016,7 +11016,7 @@
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>Jimmy Bowman</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="B321" s="2" t="inlineStr">

</xml_diff>